<commit_message>
Fill Excel result headers from event data and print communique per row
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Templates/ResultListCircuit.xlsx
+++ b/Templates/ResultListCircuit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\SmartTiming\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF84A7FD-C767-4CA3-A722-FA1FEDA984A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8393DBCF-2E95-4EF3-AE6D-5793874F421F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -322,6 +322,62 @@
   </cellStyles>
   <dxfs count="31">
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -455,62 +511,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -721,14 +721,14 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Ergebnisliste" displayName="Ergebnisliste" ref="A1:H2" insertRow="1" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17">
   <tableColumns count="8">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Platz" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Start#" dataDxfId="6"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Name, Vorname" dataDxfId="5" dataCellStyle="Standard"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Team" dataDxfId="4" dataCellStyle="Standard"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="UCI-ID" dataDxfId="3" dataCellStyle="Standard"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Zeit" dataDxfId="2" dataCellStyle="Datum"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Runden" dataDxfId="1" dataCellStyle="Datum"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Rückstand" dataDxfId="0" dataCellStyle="Standard"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Platz" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Start#" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Name, Vorname" dataDxfId="13" dataCellStyle="Standard"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Team" dataDxfId="12" dataCellStyle="Standard"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="UCI-ID" dataDxfId="11" dataCellStyle="Standard"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Zeit" dataDxfId="10" dataCellStyle="Datum"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Runden" dataDxfId="9" dataCellStyle="Datum"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Rückstand" dataDxfId="8" dataCellStyle="Standard"/>
   </tableColumns>
   <tableStyleInfo name="Aufgabenliste" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
   <extLst>
@@ -2499,53 +2499,53 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A2">
-    <cfRule type="expression" dxfId="15" priority="9">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3">
-    <cfRule type="expression" dxfId="14" priority="8">
+    <cfRule type="expression" dxfId="6" priority="8">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4">
-    <cfRule type="expression" dxfId="13" priority="7">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5">
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="4" priority="6">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6">
-    <cfRule type="expression" dxfId="11" priority="5">
+    <cfRule type="expression" dxfId="3" priority="5">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2">
-    <cfRule type="expression" dxfId="10" priority="10">
+    <cfRule type="expression" dxfId="2" priority="10">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B6">
-    <cfRule type="expression" dxfId="9" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:G2">
-    <cfRule type="expression" dxfId="8" priority="24">
+    <cfRule type="expression" dxfId="0" priority="24">
       <formula>AND(#REF!=0,#REF!&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="1.3385826771653544" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
-  <headerFooter>
-    <oddHeader>&amp;L&amp;16&amp;G&amp;C&amp;"Arial,Fett"&amp;16Offizielles Ergebnis
-Baden-Württembergische Meisterschaften Einzelzeitfahren&amp;R&amp;G</oddHeader>
-    <oddFooter>&amp;L&amp;"Arial,Standard"&amp;10Badischer Radsportverband
-Kollgium der Kommissäre&amp;C&amp;10Seite &amp;P von &amp;N&amp;R&amp;10&amp;D &amp;T</oddFooter>
+  <headerFooter scaleWithDoc="0">
+    <oddHeader>&amp;L&amp;16&amp;G&amp;C&amp;"Arial,Fett"&amp;16Offizielles &amp;14Ergebnis
+&lt;Organizer&gt; - &lt;Event-Title&gt;&amp;R&amp;G</oddHeader>
+    <oddFooter>&amp;L&amp;"Arial,Standard"&amp;12Badischer Radsport-Verband e.V.
+Kollgium der Kommissäre&amp;C&amp;"Arial,Standard"&amp;12Seite &amp;P von &amp;N&amp;R&amp;"Arial,Standard"&amp;12&amp;D &amp;T</oddFooter>
   </headerFooter>
   <legacyDrawingHF r:id="rId2"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Remember the last race type for new races.
And: Communiqué header bold and left aligned

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Templates/ResultListCircuit.xlsx
+++ b/Templates/ResultListCircuit.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\SmartTiming\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8393DBCF-2E95-4EF3-AE6D-5793874F421F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CD06C8F-DDFA-4DF3-A210-19EFBEE2C0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="24330" windowHeight="13485" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgabenliste" sheetId="1" r:id="rId1"/>
@@ -247,7 +247,7 @@
       <alignment horizontal="right" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -304,6 +304,30 @@
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -1020,232 +1044,257 @@
       <c r="G2" s="14"/>
       <c r="H2" s="15"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="14"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="14"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="14"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="14"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="14"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="14"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="14"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="14"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="14"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="14"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="14"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="14"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="14"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="14"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="14"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="14"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="14"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="14"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="14"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="14"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="14"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="14"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="14"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="23"/>
+    </row>
+    <row r="4" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="19"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="23"/>
+    </row>
+    <row r="5" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="23"/>
+    </row>
+    <row r="6" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="23"/>
+    </row>
+    <row r="7" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="23"/>
+    </row>
+    <row r="8" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="23"/>
+    </row>
+    <row r="9" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="23"/>
+    </row>
+    <row r="10" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="23"/>
+    </row>
+    <row r="11" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="23"/>
+    </row>
+    <row r="12" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="23"/>
+    </row>
+    <row r="13" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="25"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="23"/>
+    </row>
+    <row r="14" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="23"/>
+    </row>
+    <row r="15" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="20"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="23"/>
+    </row>
+    <row r="16" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="23"/>
+    </row>
+    <row r="17" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="23"/>
+    </row>
+    <row r="18" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="23"/>
+    </row>
+    <row r="19" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="23"/>
+    </row>
+    <row r="20" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="20"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="23"/>
+    </row>
+    <row r="21" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="23"/>
+    </row>
+    <row r="22" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="23"/>
+    </row>
+    <row r="23" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="23"/>
+    </row>
+    <row r="24" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="20"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="23"/>
+    </row>
+    <row r="25" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="23"/>
+    </row>
+    <row r="26" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="23"/>
+    </row>
+    <row r="27" spans="1:8" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="20"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="23"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="8"/>
@@ -1254,7 +1303,7 @@
       <c r="F28" s="17"/>
       <c r="G28" s="14"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="8"/>
@@ -1263,7 +1312,7 @@
       <c r="F29" s="17"/>
       <c r="G29" s="14"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="8"/>
@@ -1272,7 +1321,7 @@
       <c r="F30" s="17"/>
       <c r="G30" s="14"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="8"/>
@@ -1281,7 +1330,7 @@
       <c r="F31" s="17"/>
       <c r="G31" s="14"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="8"/>

</xml_diff>